<commit_message>
fix: use correct modalities in xlsx / csv header
</commit_message>
<xml_diff>
--- a/tests/eindhoven-500/reference/resultaten/werk/alle groepen/herkomsten/restdag/Pot_totaal_hoog.xlsx
+++ b/tests/eindhoven-500/reference/resultaten/werk/alle groepen/herkomsten/restdag/Pot_totaal_hoog.xlsx
@@ -14,15 +14,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Zone</t>
   </si>
   <si>
     <t>Fiets</t>
-  </si>
-  <si>
-    <t>EFiets</t>
   </si>
   <si>
     <t>Auto</t>
@@ -37,19 +34,10 @@
     <t>OV_Fiets</t>
   </si>
   <si>
-    <t>Auto_EFiets</t>
-  </si>
-  <si>
-    <t>OV_EFiets</t>
-  </si>
-  <si>
     <t>Auto_OV</t>
   </si>
   <si>
     <t>Auto_OV_Fiets</t>
-  </si>
-  <si>
-    <t>Auto_OV_EFiets</t>
   </si>
 </sst>
 </file>
@@ -381,10 +369,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L501"/>
+  <dimension ref="A1:H501"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -409,20 +397,8 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12">
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2">
         <v>1</v>
       </c>
@@ -448,7 +424,7 @@
         <v>66236</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:8">
       <c r="A3">
         <v>2</v>
       </c>
@@ -474,7 +450,7 @@
         <v>68932</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:8">
       <c r="A4">
         <v>3</v>
       </c>
@@ -500,7 +476,7 @@
         <v>63272</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:8">
       <c r="A5">
         <v>4</v>
       </c>
@@ -526,7 +502,7 @@
         <v>63272</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:8">
       <c r="A6">
         <v>5</v>
       </c>
@@ -552,7 +528,7 @@
         <v>63272</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:8">
       <c r="A7">
         <v>6</v>
       </c>
@@ -578,7 +554,7 @@
         <v>67209</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:8">
       <c r="A8">
         <v>7</v>
       </c>
@@ -604,7 +580,7 @@
         <v>67209</v>
       </c>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="1:8">
       <c r="A9">
         <v>8</v>
       </c>
@@ -630,7 +606,7 @@
         <v>65471</v>
       </c>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="1:8">
       <c r="A10">
         <v>9</v>
       </c>
@@ -656,7 +632,7 @@
         <v>67209</v>
       </c>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="1:8">
       <c r="A11">
         <v>10</v>
       </c>
@@ -682,7 +658,7 @@
         <v>67209</v>
       </c>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="1:8">
       <c r="A12">
         <v>11</v>
       </c>
@@ -708,7 +684,7 @@
         <v>63272</v>
       </c>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="1:8">
       <c r="A13">
         <v>12</v>
       </c>
@@ -734,7 +710,7 @@
         <v>68932</v>
       </c>
     </row>
-    <row r="14" spans="1:12">
+    <row r="14" spans="1:8">
       <c r="A14">
         <v>13</v>
       </c>
@@ -760,7 +736,7 @@
         <v>63272</v>
       </c>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="1:8">
       <c r="A15">
         <v>14</v>
       </c>
@@ -786,7 +762,7 @@
         <v>67209</v>
       </c>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="1:8">
       <c r="A16">
         <v>15</v>
       </c>

</xml_diff>